<commit_message>
added game from 2026-09-03
</commit_message>
<xml_diff>
--- a/backend/TerraformingMarsTotalStats.xlsx
+++ b/backend/TerraformingMarsTotalStats.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="25"/>
   </bookViews>
   <sheets>
     <sheet name="09.10.2025" sheetId="1" state="visible" r:id="rId3"/>
@@ -33,6 +33,7 @@
     <sheet name="02.07.2026" sheetId="23" state="visible" r:id="rId25"/>
     <sheet name="09.07.2026" sheetId="24" state="visible" r:id="rId26"/>
     <sheet name="16.07.2026" sheetId="25" state="visible" r:id="rId27"/>
+    <sheet name="03.09.2026" sheetId="26" state="visible" r:id="rId28"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="41">
   <si>
     <t xml:space="preserve">players</t>
   </si>
@@ -270,37 +271,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -3232,6 +3233,173 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="C2" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="D2" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="F2" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="G2" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="H2" s="0" t="n">
+        <v>107</v>
+      </c>
+      <c r="J2" s="0" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="C3" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="F3" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="G3" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="H3" s="0" t="n">
+        <v>102</v>
+      </c>
+      <c r="J3" s="0" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="C4" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="E4" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="F4" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="G4" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="H4" s="0" t="n">
+        <v>99</v>
+      </c>
+      <c r="J4" s="0" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="C5" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="E5" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="H5" s="0" t="n">
+        <v>79</v>
+      </c>
+      <c r="J5" s="0" t="s">
+        <v>31</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Standard"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Standard"&amp;12Seite &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">

</xml_diff>